<commit_message>
feat: implement configurable match side mirroring with default White-on-left layout
</commit_message>
<xml_diff>
--- a/playoffs-example-large.xlsx
+++ b/playoffs-example-large.xlsx
@@ -678,13 +678,13 @@
     <t>Match 1</t>
   </si>
   <si>
+    <t>White</t>
+  </si>
+  <si>
+    <t>vs</t>
+  </si>
+  <si>
     <t>Red</t>
-  </si>
-  <si>
-    <t>vs</t>
-  </si>
-  <si>
-    <t>White</t>
   </si>
   <si>
     <t>1.</t>
@@ -5847,28 +5847,28 @@
       <c r="O3" s="20"/>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D4" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G4" s="30" t="s">
+      <c r="G4" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I4" s="29" t="s">
+      <c r="I4" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L4" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O4" s="30" t="s">
+      <c r="O4" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="str">
-        <f>'data'!$B$6</f>
+        <f>'data'!$B$35</f>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="28"/>
@@ -5876,10 +5876,10 @@
       <c r="E5" s="28"/>
       <c r="F5" s="28"/>
       <c r="G5" s="28" t="str">
-        <f>'data'!$B$35</f>
+        <f>'data'!$B$6</f>
       </c>
       <c r="I5" s="28" t="str">
-        <f>'data'!$B$37</f>
+        <f>'data'!$B$38</f>
       </c>
       <c r="J5" s="28"/>
       <c r="K5" s="28"/>
@@ -5887,7 +5887,7 @@
       <c r="M5" s="28"/>
       <c r="N5" s="28"/>
       <c r="O5" s="28" t="str">
-        <f>'data'!$B$38</f>
+        <f>'data'!$B$37</f>
       </c>
     </row>
     <row r="7">
@@ -5931,28 +5931,28 @@
       <c r="O11" s="20"/>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D12" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G12" s="30" t="s">
+      <c r="G12" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I12" s="29" t="s">
+      <c r="I12" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L12" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O12" s="30" t="s">
+      <c r="O12" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="str">
-        <f>'data'!$B$40</f>
+        <f>'data'!$B$41</f>
       </c>
       <c r="B13" s="28"/>
       <c r="C13" s="28"/>
@@ -5960,10 +5960,10 @@
       <c r="E13" s="28"/>
       <c r="F13" s="28"/>
       <c r="G13" s="28" t="str">
-        <f>'data'!$B$41</f>
+        <f>'data'!$B$40</f>
       </c>
       <c r="I13" s="28" t="str">
-        <f>'data'!$B$17</f>
+        <f>'data'!$B$18</f>
       </c>
       <c r="J13" s="28"/>
       <c r="K13" s="28"/>
@@ -5971,7 +5971,7 @@
       <c r="M13" s="28"/>
       <c r="N13" s="28"/>
       <c r="O13" s="28" t="str">
-        <f>'data'!$B$18</f>
+        <f>'data'!$B$17</f>
       </c>
     </row>
     <row r="15">
@@ -6015,28 +6015,28 @@
       <c r="O19" s="20"/>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D20" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G20" s="30" t="s">
+      <c r="G20" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I20" s="29" t="s">
+      <c r="I20" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L20" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O20" s="30" t="s">
+      <c r="O20" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="str">
-        <f>'data'!$B$20</f>
+        <f>'data'!$B$21</f>
       </c>
       <c r="B21" s="28"/>
       <c r="C21" s="28"/>
@@ -6044,10 +6044,10 @@
       <c r="E21" s="28"/>
       <c r="F21" s="28"/>
       <c r="G21" s="28" t="str">
-        <f>'data'!$B$21</f>
+        <f>'data'!$B$20</f>
       </c>
       <c r="I21" s="28" t="str">
-        <f>'data'!$B$23</f>
+        <f>'data'!$B$24</f>
       </c>
       <c r="J21" s="28"/>
       <c r="K21" s="28"/>
@@ -6055,7 +6055,7 @@
       <c r="M21" s="28"/>
       <c r="N21" s="28"/>
       <c r="O21" s="28" t="str">
-        <f>'data'!$B$24</f>
+        <f>'data'!$B$23</f>
       </c>
     </row>
     <row r="23">
@@ -6099,28 +6099,28 @@
       <c r="O27" s="20"/>
     </row>
     <row r="28">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D28" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G28" s="30" t="s">
+      <c r="G28" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I28" s="29" t="s">
+      <c r="I28" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L28" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O28" s="30" t="s">
+      <c r="O28" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="str">
-        <f>'data'!$B$28</f>
+        <f>'data'!$B$29</f>
       </c>
       <c r="B29" s="28"/>
       <c r="C29" s="28"/>
@@ -6128,10 +6128,10 @@
       <c r="E29" s="28"/>
       <c r="F29" s="28"/>
       <c r="G29" s="28" t="str">
-        <f>'data'!$B$29</f>
+        <f>'data'!$B$28</f>
       </c>
       <c r="I29" s="28" t="str">
-        <f>'data'!$B$31</f>
+        <f>'data'!$B$32</f>
       </c>
       <c r="J29" s="28"/>
       <c r="K29" s="28"/>
@@ -6139,7 +6139,7 @@
       <c r="M29" s="28"/>
       <c r="N29" s="28"/>
       <c r="O29" s="28" t="str">
-        <f>'data'!$B$32</f>
+        <f>'data'!$B$31</f>
       </c>
     </row>
     <row r="31">
@@ -6183,28 +6183,28 @@
       <c r="O35" s="20"/>
     </row>
     <row r="36">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D36" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G36" s="30" t="s">
+      <c r="G36" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I36" s="29" t="s">
+      <c r="I36" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L36" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O36" s="30" t="s">
+      <c r="O36" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="str">
-        <f>'data'!$B$34</f>
+        <f>'data'!$B$35</f>
       </c>
       <c r="B37" s="28"/>
       <c r="C37" s="28"/>
@@ -6212,10 +6212,10 @@
       <c r="E37" s="28"/>
       <c r="F37" s="28"/>
       <c r="G37" s="28" t="str">
-        <f>'data'!$B$35</f>
+        <f>'data'!$B$34</f>
       </c>
       <c r="I37" s="28" t="str">
-        <f>'data'!$B$37</f>
+        <f>'data'!$B$38</f>
       </c>
       <c r="J37" s="28"/>
       <c r="K37" s="28"/>
@@ -6223,7 +6223,7 @@
       <c r="M37" s="28"/>
       <c r="N37" s="28"/>
       <c r="O37" s="28" t="str">
-        <f>'data'!$B$38</f>
+        <f>'data'!$B$37</f>
       </c>
     </row>
     <row r="39">
@@ -6267,28 +6267,28 @@
       <c r="O43" s="20"/>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="s">
+      <c r="A44" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D44" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G44" s="30" t="s">
+      <c r="G44" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I44" s="29" t="s">
+      <c r="I44" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L44" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O44" s="30" t="s">
+      <c r="O44" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="28" t="str">
-        <f>'data'!$B$40</f>
+        <f>'data'!$B$41</f>
       </c>
       <c r="B45" s="28"/>
       <c r="C45" s="28"/>
@@ -6296,10 +6296,10 @@
       <c r="E45" s="28"/>
       <c r="F45" s="28"/>
       <c r="G45" s="28" t="str">
-        <f>'data'!$B$41</f>
+        <f>'data'!$B$40</f>
       </c>
       <c r="I45" s="28" t="str">
-        <f>'data'!$B$43</f>
+        <f>'data'!$B$44</f>
       </c>
       <c r="J45" s="28"/>
       <c r="K45" s="28"/>
@@ -6307,7 +6307,7 @@
       <c r="M45" s="28"/>
       <c r="N45" s="28"/>
       <c r="O45" s="28" t="str">
-        <f>'data'!$B$44</f>
+        <f>'data'!$B$43</f>
       </c>
     </row>
     <row r="47">
@@ -6351,28 +6351,28 @@
       <c r="O51" s="20"/>
     </row>
     <row r="52">
-      <c r="A52" s="29" t="s">
+      <c r="A52" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D52" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G52" s="30" t="s">
+      <c r="G52" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I52" s="29" t="s">
+      <c r="I52" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L52" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O52" s="30" t="s">
+      <c r="O52" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="28" t="str">
-        <f>'data'!$B$46</f>
+        <f>'data'!$B$47</f>
       </c>
       <c r="B53" s="28"/>
       <c r="C53" s="28"/>
@@ -6380,10 +6380,10 @@
       <c r="E53" s="28"/>
       <c r="F53" s="28"/>
       <c r="G53" s="28" t="str">
-        <f>'data'!$B$47</f>
+        <f>'data'!$B$46</f>
       </c>
       <c r="I53" s="28" t="str">
-        <f>'data'!$B$51</f>
+        <f>'data'!$B$52</f>
       </c>
       <c r="J53" s="28"/>
       <c r="K53" s="28"/>
@@ -6391,7 +6391,7 @@
       <c r="M53" s="28"/>
       <c r="N53" s="28"/>
       <c r="O53" s="28" t="str">
-        <f>'data'!$B$52</f>
+        <f>'data'!$B$51</f>
       </c>
     </row>
     <row r="55">
@@ -6435,28 +6435,28 @@
       <c r="O59" s="20"/>
     </row>
     <row r="60">
-      <c r="A60" s="29" t="s">
+      <c r="A60" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D60" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G60" s="30" t="s">
+      <c r="G60" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I60" s="29" t="s">
+      <c r="I60" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L60" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O60" s="30" t="s">
+      <c r="O60" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="28" t="str">
-        <f>'data'!$B$54</f>
+        <f>'data'!$B$55</f>
       </c>
       <c r="B61" s="28"/>
       <c r="C61" s="28"/>
@@ -6464,10 +6464,10 @@
       <c r="E61" s="28"/>
       <c r="F61" s="28"/>
       <c r="G61" s="28" t="str">
-        <f>'data'!$B$55</f>
+        <f>'data'!$B$54</f>
       </c>
       <c r="I61" s="28" t="str">
-        <f>'data'!$B$57</f>
+        <f>'data'!$B$58</f>
       </c>
       <c r="J61" s="28"/>
       <c r="K61" s="28"/>
@@ -6475,7 +6475,7 @@
       <c r="M61" s="28"/>
       <c r="N61" s="28"/>
       <c r="O61" s="28" t="str">
-        <f>'data'!$B$58</f>
+        <f>'data'!$B$57</f>
       </c>
     </row>
     <row r="63">
@@ -6519,28 +6519,28 @@
       <c r="O67" s="20"/>
     </row>
     <row r="68">
-      <c r="A68" s="29" t="s">
+      <c r="A68" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D68" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G68" s="30" t="s">
+      <c r="G68" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I68" s="29" t="s">
+      <c r="I68" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L68" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O68" s="30" t="s">
+      <c r="O68" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="28" t="str">
-        <f>'data'!$B$60</f>
+        <f>'data'!$B$61</f>
       </c>
       <c r="B69" s="28"/>
       <c r="C69" s="28"/>
@@ -6548,10 +6548,10 @@
       <c r="E69" s="28"/>
       <c r="F69" s="28"/>
       <c r="G69" s="28" t="str">
-        <f>'data'!$B$61</f>
+        <f>'data'!$B$60</f>
       </c>
       <c r="I69" s="28" t="str">
-        <f>'data'!$B$63</f>
+        <f>'data'!$B$64</f>
       </c>
       <c r="J69" s="28"/>
       <c r="K69" s="28"/>
@@ -6559,7 +6559,7 @@
       <c r="M69" s="28"/>
       <c r="N69" s="28"/>
       <c r="O69" s="28" t="str">
-        <f>'data'!$B$64</f>
+        <f>'data'!$B$63</f>
       </c>
     </row>
     <row r="71">
@@ -6603,28 +6603,28 @@
       <c r="O75" s="20"/>
     </row>
     <row r="76">
-      <c r="A76" s="29" t="s">
+      <c r="A76" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D76" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G76" s="30" t="s">
+      <c r="G76" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I76" s="29" t="s">
+      <c r="I76" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L76" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O76" s="30" t="s">
+      <c r="O76" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="28" t="str">
-        <f>'data'!$B$66</f>
+        <f>'data'!$B$67</f>
       </c>
       <c r="B77" s="28"/>
       <c r="C77" s="28"/>
@@ -6632,10 +6632,10 @@
       <c r="E77" s="28"/>
       <c r="F77" s="28"/>
       <c r="G77" s="28" t="str">
-        <f>'data'!$B$67</f>
+        <f>'data'!$B$66</f>
       </c>
       <c r="I77" s="28" t="str">
-        <f>'data'!$B$69</f>
+        <f>'data'!$B$74</f>
       </c>
       <c r="J77" s="28"/>
       <c r="K77" s="28"/>
@@ -6643,7 +6643,7 @@
       <c r="M77" s="28"/>
       <c r="N77" s="28"/>
       <c r="O77" s="28" t="str">
-        <f>'data'!$B$74</f>
+        <f>'data'!$B$69</f>
       </c>
     </row>
     <row r="79">
@@ -6687,28 +6687,28 @@
       <c r="O83" s="20"/>
     </row>
     <row r="84">
-      <c r="A84" s="29" t="s">
+      <c r="A84" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D84" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G84" s="30" t="s">
+      <c r="G84" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I84" s="29" t="s">
+      <c r="I84" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L84" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O84" s="30" t="s">
+      <c r="O84" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="28" t="str">
-        <f>'data'!$B$74</f>
+        <f>'data'!$B$75</f>
       </c>
       <c r="B85" s="28"/>
       <c r="C85" s="28"/>
@@ -6716,10 +6716,10 @@
       <c r="E85" s="28"/>
       <c r="F85" s="28"/>
       <c r="G85" s="28" t="str">
-        <f>'data'!$B$75</f>
+        <f>'data'!$B$74</f>
       </c>
       <c r="I85" s="28" t="str">
-        <f>'data'!$B$77</f>
+        <f>'data'!$B$78</f>
       </c>
       <c r="J85" s="28"/>
       <c r="K85" s="28"/>
@@ -6727,7 +6727,7 @@
       <c r="M85" s="28"/>
       <c r="N85" s="28"/>
       <c r="O85" s="28" t="str">
-        <f>'data'!$B$78</f>
+        <f>'data'!$B$77</f>
       </c>
     </row>
     <row r="87">
@@ -6771,28 +6771,28 @@
       <c r="O91" s="20"/>
     </row>
     <row r="92">
-      <c r="A92" s="29" t="s">
+      <c r="A92" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D92" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G92" s="30" t="s">
+      <c r="G92" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I92" s="29" t="s">
+      <c r="I92" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L92" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O92" s="30" t="s">
+      <c r="O92" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="28" t="str">
-        <f>'data'!$B$80</f>
+        <f>'data'!$B$81</f>
       </c>
       <c r="B93" s="28"/>
       <c r="C93" s="28"/>
@@ -6800,10 +6800,10 @@
       <c r="E93" s="28"/>
       <c r="F93" s="28"/>
       <c r="G93" s="28" t="str">
-        <f>'data'!$B$81</f>
+        <f>'data'!$B$80</f>
       </c>
       <c r="I93" s="28" t="str">
-        <f>'data'!$B$83</f>
+        <f>'data'!$B$84</f>
       </c>
       <c r="J93" s="28"/>
       <c r="K93" s="28"/>
@@ -6811,7 +6811,7 @@
       <c r="M93" s="28"/>
       <c r="N93" s="28"/>
       <c r="O93" s="28" t="str">
-        <f>'data'!$B$84</f>
+        <f>'data'!$B$83</f>
       </c>
     </row>
     <row r="95">
@@ -6855,28 +6855,28 @@
       <c r="O99" s="20"/>
     </row>
     <row r="100">
-      <c r="A100" s="29" t="s">
+      <c r="A100" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D100" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G100" s="30" t="s">
+      <c r="G100" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I100" s="29" t="s">
+      <c r="I100" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L100" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O100" s="30" t="s">
+      <c r="O100" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="28" t="str">
-        <f>'data'!$B$86</f>
+        <f>'data'!$B$87</f>
       </c>
       <c r="B101" s="28"/>
       <c r="C101" s="28"/>
@@ -6884,10 +6884,10 @@
       <c r="E101" s="28"/>
       <c r="F101" s="28"/>
       <c r="G101" s="28" t="str">
-        <f>'data'!$B$87</f>
+        <f>'data'!$B$86</f>
       </c>
       <c r="I101" s="28" t="str">
-        <f>'data'!$B$89</f>
+        <f>'data'!$B$90</f>
       </c>
       <c r="J101" s="28"/>
       <c r="K101" s="28"/>
@@ -6895,7 +6895,7 @@
       <c r="M101" s="28"/>
       <c r="N101" s="28"/>
       <c r="O101" s="28" t="str">
-        <f>'data'!$B$90</f>
+        <f>'data'!$B$89</f>
       </c>
     </row>
     <row r="103">
@@ -6930,19 +6930,19 @@
       <c r="G107" s="20"/>
     </row>
     <row r="108">
-      <c r="A108" s="29" t="s">
+      <c r="A108" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D108" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G108" s="30" t="s">
+      <c r="G108" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="28" t="str">
-        <f>'data'!$B$92</f>
+        <f>'data'!$B$93</f>
       </c>
       <c r="B109" s="28"/>
       <c r="C109" s="28"/>
@@ -6950,7 +6950,7 @@
       <c r="E109" s="28"/>
       <c r="F109" s="28"/>
       <c r="G109" s="28" t="str">
-        <f>'data'!$B$93</f>
+        <f>'data'!$B$92</f>
       </c>
     </row>
     <row r="111">
@@ -7005,28 +7005,28 @@
       <c r="O122" s="20"/>
     </row>
     <row r="123">
-      <c r="A123" s="29" t="s">
+      <c r="A123" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D123" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G123" s="30" t="s">
+      <c r="G123" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I123" s="29" t="s">
+      <c r="I123" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L123" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O123" s="30" t="s">
+      <c r="O123" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="28" t="str">
-        <f>'data'!$B$32</f>
+        <f>'data'!$B$33</f>
       </c>
       <c r="B124" s="28"/>
       <c r="C124" s="28"/>
@@ -7034,10 +7034,10 @@
       <c r="E124" s="28"/>
       <c r="F124" s="28"/>
       <c r="G124" s="28" t="str">
-        <f>'data'!$B$33</f>
+        <f>'data'!$B$32</f>
       </c>
       <c r="I124" s="28" t="str">
-        <f>'data'!$B$34</f>
+        <f>CONCATENATE("M 1 ",'Elimination Matches'!G7)</f>
       </c>
       <c r="J124" s="28"/>
       <c r="K124" s="28"/>
@@ -7045,7 +7045,7 @@
       <c r="M124" s="28"/>
       <c r="N124" s="28"/>
       <c r="O124" s="28" t="str">
-        <f>CONCATENATE("M 1 ",'Elimination Matches'!G7)</f>
+        <f>'data'!$B$34</f>
       </c>
     </row>
     <row r="126">
@@ -7089,28 +7089,28 @@
       <c r="O130" s="20"/>
     </row>
     <row r="131">
-      <c r="A131" s="29" t="s">
+      <c r="A131" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D131" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G131" s="30" t="s">
+      <c r="G131" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I131" s="29" t="s">
+      <c r="I131" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L131" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O131" s="30" t="s">
+      <c r="O131" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="28" t="str">
-        <f>'data'!$B$36</f>
+        <f>CONCATENATE("M 2 ",'Elimination Matches'!O7)</f>
       </c>
       <c r="B132" s="28"/>
       <c r="C132" s="28"/>
@@ -7118,10 +7118,10 @@
       <c r="E132" s="28"/>
       <c r="F132" s="28"/>
       <c r="G132" s="28" t="str">
-        <f>CONCATENATE("M 2 ",'Elimination Matches'!O7)</f>
+        <f>'data'!$B$36</f>
       </c>
       <c r="I132" s="28" t="str">
-        <f>'data'!$B$39</f>
+        <f>CONCATENATE("M 3 ",'Elimination Matches'!G15)</f>
       </c>
       <c r="J132" s="28"/>
       <c r="K132" s="28"/>
@@ -7129,7 +7129,7 @@
       <c r="M132" s="28"/>
       <c r="N132" s="28"/>
       <c r="O132" s="28" t="str">
-        <f>CONCATENATE("M 3 ",'Elimination Matches'!G15)</f>
+        <f>'data'!$B$39</f>
       </c>
     </row>
     <row r="134">
@@ -7173,28 +7173,28 @@
       <c r="O138" s="20"/>
     </row>
     <row r="139">
-      <c r="A139" s="29" t="s">
+      <c r="A139" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D139" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G139" s="30" t="s">
+      <c r="G139" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I139" s="29" t="s">
+      <c r="I139" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L139" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O139" s="30" t="s">
+      <c r="O139" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="28" t="str">
-        <f>'data'!$B$42</f>
+        <f>'data'!$B$43</f>
       </c>
       <c r="B140" s="28"/>
       <c r="C140" s="28"/>
@@ -7202,10 +7202,10 @@
       <c r="E140" s="28"/>
       <c r="F140" s="28"/>
       <c r="G140" s="28" t="str">
-        <f>'data'!$B$43</f>
+        <f>'data'!$B$42</f>
       </c>
       <c r="I140" s="28" t="str">
-        <f>'data'!$B$16</f>
+        <f>CONCATENATE("M 4 ",'Elimination Matches'!O15)</f>
       </c>
       <c r="J140" s="28"/>
       <c r="K140" s="28"/>
@@ -7213,7 +7213,7 @@
       <c r="M140" s="28"/>
       <c r="N140" s="28"/>
       <c r="O140" s="28" t="str">
-        <f>CONCATENATE("M 4 ",'Elimination Matches'!O15)</f>
+        <f>'data'!$B$16</f>
       </c>
     </row>
     <row r="142">
@@ -7257,28 +7257,28 @@
       <c r="O146" s="20"/>
     </row>
     <row r="147">
-      <c r="A147" s="29" t="s">
+      <c r="A147" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D147" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G147" s="30" t="s">
+      <c r="G147" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I147" s="29" t="s">
+      <c r="I147" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L147" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O147" s="30" t="s">
+      <c r="O147" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="28" t="str">
-        <f>'data'!$B$30</f>
+        <f>CONCATENATE("M 5 ",'Elimination Matches'!G23)</f>
       </c>
       <c r="B148" s="28"/>
       <c r="C148" s="28"/>
@@ -7286,10 +7286,10 @@
       <c r="E148" s="28"/>
       <c r="F148" s="28"/>
       <c r="G148" s="28" t="str">
-        <f>CONCATENATE("M 5 ",'Elimination Matches'!G23)</f>
+        <f>'data'!$B$30</f>
       </c>
       <c r="I148" s="28" t="str">
-        <f>'data'!$B$22</f>
+        <f>CONCATENATE("M 6 ",'Elimination Matches'!O23)</f>
       </c>
       <c r="J148" s="28"/>
       <c r="K148" s="28"/>
@@ -7297,7 +7297,7 @@
       <c r="M148" s="28"/>
       <c r="N148" s="28"/>
       <c r="O148" s="28" t="str">
-        <f>CONCATENATE("M 6 ",'Elimination Matches'!O23)</f>
+        <f>'data'!$B$22</f>
       </c>
     </row>
     <row r="150">
@@ -7341,28 +7341,28 @@
       <c r="O154" s="20"/>
     </row>
     <row r="155">
-      <c r="A155" s="29" t="s">
+      <c r="A155" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D155" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G155" s="30" t="s">
+      <c r="G155" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I155" s="29" t="s">
+      <c r="I155" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L155" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O155" s="30" t="s">
+      <c r="O155" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="28" t="str">
-        <f>'data'!$B$25</f>
+        <f>'data'!$B$26</f>
       </c>
       <c r="B156" s="28"/>
       <c r="C156" s="28"/>
@@ -7370,10 +7370,10 @@
       <c r="E156" s="28"/>
       <c r="F156" s="28"/>
       <c r="G156" s="28" t="str">
-        <f>'data'!$B$26</f>
+        <f>'data'!$B$25</f>
       </c>
       <c r="I156" s="28" t="str">
-        <f>'data'!$B$27</f>
+        <f>CONCATENATE("M 7 ",'Elimination Matches'!G31)</f>
       </c>
       <c r="J156" s="28"/>
       <c r="K156" s="28"/>
@@ -7381,7 +7381,7 @@
       <c r="M156" s="28"/>
       <c r="N156" s="28"/>
       <c r="O156" s="28" t="str">
-        <f>CONCATENATE("M 7 ",'Elimination Matches'!G31)</f>
+        <f>'data'!$B$27</f>
       </c>
     </row>
     <row r="158">
@@ -7425,28 +7425,28 @@
       <c r="O162" s="20"/>
     </row>
     <row r="163">
-      <c r="A163" s="29" t="s">
+      <c r="A163" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D163" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G163" s="30" t="s">
+      <c r="G163" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I163" s="29" t="s">
+      <c r="I163" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L163" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O163" s="30" t="s">
+      <c r="O163" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="28" t="str">
-        <f>'data'!$B$30</f>
+        <f>CONCATENATE("M 8 ",'Elimination Matches'!O31)</f>
       </c>
       <c r="B164" s="28"/>
       <c r="C164" s="28"/>
@@ -7454,10 +7454,10 @@
       <c r="E164" s="28"/>
       <c r="F164" s="28"/>
       <c r="G164" s="28" t="str">
-        <f>CONCATENATE("M 8 ",'Elimination Matches'!O31)</f>
+        <f>'data'!$B$30</f>
       </c>
       <c r="I164" s="28" t="str">
-        <f>'data'!$B$33</f>
+        <f>CONCATENATE("M 9 ",'Elimination Matches'!G39)</f>
       </c>
       <c r="J164" s="28"/>
       <c r="K164" s="28"/>
@@ -7465,7 +7465,7 @@
       <c r="M164" s="28"/>
       <c r="N164" s="28"/>
       <c r="O164" s="28" t="str">
-        <f>CONCATENATE("M 9 ",'Elimination Matches'!G39)</f>
+        <f>'data'!$B$33</f>
       </c>
     </row>
     <row r="166">
@@ -7509,28 +7509,28 @@
       <c r="O170" s="20"/>
     </row>
     <row r="171">
-      <c r="A171" s="29" t="s">
+      <c r="A171" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D171" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G171" s="30" t="s">
+      <c r="G171" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I171" s="29" t="s">
+      <c r="I171" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L171" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O171" s="30" t="s">
+      <c r="O171" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="28" t="str">
-        <f>'data'!$B$36</f>
+        <f>CONCATENATE("M 10 ",'Elimination Matches'!O39)</f>
       </c>
       <c r="B172" s="28"/>
       <c r="C172" s="28"/>
@@ -7538,10 +7538,10 @@
       <c r="E172" s="28"/>
       <c r="F172" s="28"/>
       <c r="G172" s="28" t="str">
-        <f>CONCATENATE("M 10 ",'Elimination Matches'!O39)</f>
+        <f>'data'!$B$36</f>
       </c>
       <c r="I172" s="28" t="str">
-        <f>'data'!$B$39</f>
+        <f>CONCATENATE("M 11 ",'Elimination Matches'!G47)</f>
       </c>
       <c r="J172" s="28"/>
       <c r="K172" s="28"/>
@@ -7549,7 +7549,7 @@
       <c r="M172" s="28"/>
       <c r="N172" s="28"/>
       <c r="O172" s="28" t="str">
-        <f>CONCATENATE("M 11 ",'Elimination Matches'!G47)</f>
+        <f>'data'!$B$39</f>
       </c>
     </row>
     <row r="174">
@@ -7593,28 +7593,28 @@
       <c r="O178" s="20"/>
     </row>
     <row r="179">
-      <c r="A179" s="29" t="s">
+      <c r="A179" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D179" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G179" s="30" t="s">
+      <c r="G179" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I179" s="29" t="s">
+      <c r="I179" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L179" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O179" s="30" t="s">
+      <c r="O179" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="28" t="str">
-        <f>'data'!$B$42</f>
+        <f>CONCATENATE("M 12 ",'Elimination Matches'!O47)</f>
       </c>
       <c r="B180" s="28"/>
       <c r="C180" s="28"/>
@@ -7622,10 +7622,10 @@
       <c r="E180" s="28"/>
       <c r="F180" s="28"/>
       <c r="G180" s="28" t="str">
-        <f>CONCATENATE("M 12 ",'Elimination Matches'!O47)</f>
+        <f>'data'!$B$42</f>
       </c>
       <c r="I180" s="28" t="str">
-        <f>'data'!$B$45</f>
+        <f>CONCATENATE("M 13 ",'Elimination Matches'!G55)</f>
       </c>
       <c r="J180" s="28"/>
       <c r="K180" s="28"/>
@@ -7633,7 +7633,7 @@
       <c r="M180" s="28"/>
       <c r="N180" s="28"/>
       <c r="O180" s="28" t="str">
-        <f>CONCATENATE("M 13 ",'Elimination Matches'!G55)</f>
+        <f>'data'!$B$45</f>
       </c>
     </row>
     <row r="182">
@@ -7677,28 +7677,28 @@
       <c r="O186" s="20"/>
     </row>
     <row r="187">
-      <c r="A187" s="29" t="s">
+      <c r="A187" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D187" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G187" s="30" t="s">
+      <c r="G187" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I187" s="29" t="s">
+      <c r="I187" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L187" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O187" s="30" t="s">
+      <c r="O187" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="28" t="str">
-        <f>'data'!$B$48</f>
+        <f>'data'!$B$49</f>
       </c>
       <c r="B188" s="28"/>
       <c r="C188" s="28"/>
@@ -7706,10 +7706,10 @@
       <c r="E188" s="28"/>
       <c r="F188" s="28"/>
       <c r="G188" s="28" t="str">
-        <f>'data'!$B$49</f>
+        <f>'data'!$B$48</f>
       </c>
       <c r="I188" s="28" t="str">
-        <f>'data'!$B$50</f>
+        <f>CONCATENATE("M 14 ",'Elimination Matches'!O55)</f>
       </c>
       <c r="J188" s="28"/>
       <c r="K188" s="28"/>
@@ -7717,7 +7717,7 @@
       <c r="M188" s="28"/>
       <c r="N188" s="28"/>
       <c r="O188" s="28" t="str">
-        <f>CONCATENATE("M 14 ",'Elimination Matches'!O55)</f>
+        <f>'data'!$B$50</f>
       </c>
     </row>
     <row r="190">
@@ -7761,28 +7761,28 @@
       <c r="O194" s="20"/>
     </row>
     <row r="195">
-      <c r="A195" s="29" t="s">
+      <c r="A195" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D195" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G195" s="30" t="s">
+      <c r="G195" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I195" s="29" t="s">
+      <c r="I195" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L195" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O195" s="30" t="s">
+      <c r="O195" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="28" t="str">
-        <f>'data'!$B$53</f>
+        <f>CONCATENATE("M 15 ",'Elimination Matches'!G63)</f>
       </c>
       <c r="B196" s="28"/>
       <c r="C196" s="28"/>
@@ -7790,10 +7790,10 @@
       <c r="E196" s="28"/>
       <c r="F196" s="28"/>
       <c r="G196" s="28" t="str">
-        <f>CONCATENATE("M 15 ",'Elimination Matches'!G63)</f>
+        <f>'data'!$B$53</f>
       </c>
       <c r="I196" s="28" t="str">
-        <f>'data'!$B$56</f>
+        <f>CONCATENATE("M 16 ",'Elimination Matches'!O63)</f>
       </c>
       <c r="J196" s="28"/>
       <c r="K196" s="28"/>
@@ -7801,7 +7801,7 @@
       <c r="M196" s="28"/>
       <c r="N196" s="28"/>
       <c r="O196" s="28" t="str">
-        <f>CONCATENATE("M 16 ",'Elimination Matches'!O63)</f>
+        <f>'data'!$B$56</f>
       </c>
     </row>
     <row r="198">
@@ -7845,28 +7845,28 @@
       <c r="O202" s="20"/>
     </row>
     <row r="203">
-      <c r="A203" s="29" t="s">
+      <c r="A203" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D203" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G203" s="30" t="s">
+      <c r="G203" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I203" s="29" t="s">
+      <c r="I203" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L203" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O203" s="30" t="s">
+      <c r="O203" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="28" t="str">
-        <f>'data'!$B$81</f>
+        <f>CONCATENATE("M 17 ",'Elimination Matches'!G71)</f>
       </c>
       <c r="B204" s="28"/>
       <c r="C204" s="28"/>
@@ -7874,10 +7874,10 @@
       <c r="E204" s="28"/>
       <c r="F204" s="28"/>
       <c r="G204" s="28" t="str">
-        <f>CONCATENATE("M 17 ",'Elimination Matches'!G71)</f>
+        <f>'data'!$B$81</f>
       </c>
       <c r="I204" s="28" t="str">
-        <f>'data'!$B$62</f>
+        <f>CONCATENATE("M 18 ",'Elimination Matches'!O71)</f>
       </c>
       <c r="J204" s="28"/>
       <c r="K204" s="28"/>
@@ -7885,7 +7885,7 @@
       <c r="M204" s="28"/>
       <c r="N204" s="28"/>
       <c r="O204" s="28" t="str">
-        <f>CONCATENATE("M 18 ",'Elimination Matches'!O71)</f>
+        <f>'data'!$B$62</f>
       </c>
     </row>
     <row r="206">
@@ -7929,28 +7929,28 @@
       <c r="O210" s="20"/>
     </row>
     <row r="211">
-      <c r="A211" s="29" t="s">
+      <c r="A211" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D211" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G211" s="30" t="s">
+      <c r="G211" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I211" s="29" t="s">
+      <c r="I211" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L211" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O211" s="30" t="s">
+      <c r="O211" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="28" t="str">
-        <f>'data'!$B$65</f>
+        <f>CONCATENATE("M 19 ",'Elimination Matches'!G79)</f>
       </c>
       <c r="B212" s="28"/>
       <c r="C212" s="28"/>
@@ -7958,10 +7958,10 @@
       <c r="E212" s="28"/>
       <c r="F212" s="28"/>
       <c r="G212" s="28" t="str">
-        <f>CONCATENATE("M 19 ",'Elimination Matches'!G79)</f>
+        <f>'data'!$B$65</f>
       </c>
       <c r="I212" s="28" t="str">
-        <f>'data'!$B$68</f>
+        <f>CONCATENATE("M 20 ",'Elimination Matches'!O79)</f>
       </c>
       <c r="J212" s="28"/>
       <c r="K212" s="28"/>
@@ -7969,7 +7969,7 @@
       <c r="M212" s="28"/>
       <c r="N212" s="28"/>
       <c r="O212" s="28" t="str">
-        <f>CONCATENATE("M 20 ",'Elimination Matches'!O79)</f>
+        <f>'data'!$B$68</f>
       </c>
     </row>
     <row r="214">
@@ -8013,28 +8013,28 @@
       <c r="O218" s="20"/>
     </row>
     <row r="219">
-      <c r="A219" s="29" t="s">
+      <c r="A219" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D219" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G219" s="30" t="s">
+      <c r="G219" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I219" s="29" t="s">
+      <c r="I219" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L219" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O219" s="30" t="s">
+      <c r="O219" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="28" t="str">
-        <f>'data'!$B$88</f>
+        <f>'data'!$B$72</f>
       </c>
       <c r="B220" s="28"/>
       <c r="C220" s="28"/>
@@ -8042,10 +8042,10 @@
       <c r="E220" s="28"/>
       <c r="F220" s="28"/>
       <c r="G220" s="28" t="str">
-        <f>'data'!$B$72</f>
+        <f>'data'!$B$88</f>
       </c>
       <c r="I220" s="28" t="str">
-        <f>'data'!$B$73</f>
+        <f>CONCATENATE("M 21 ",'Elimination Matches'!G87)</f>
       </c>
       <c r="J220" s="28"/>
       <c r="K220" s="28"/>
@@ -8053,7 +8053,7 @@
       <c r="M220" s="28"/>
       <c r="N220" s="28"/>
       <c r="O220" s="28" t="str">
-        <f>CONCATENATE("M 21 ",'Elimination Matches'!G87)</f>
+        <f>'data'!$B$73</f>
       </c>
     </row>
     <row r="222">
@@ -8097,28 +8097,28 @@
       <c r="O226" s="20"/>
     </row>
     <row r="227">
-      <c r="A227" s="29" t="s">
+      <c r="A227" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D227" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G227" s="30" t="s">
+      <c r="G227" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I227" s="29" t="s">
+      <c r="I227" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L227" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O227" s="30" t="s">
+      <c r="O227" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="28" t="str">
-        <f>'data'!$B$76</f>
+        <f>CONCATENATE("M 22 ",'Elimination Matches'!O87)</f>
       </c>
       <c r="B228" s="28"/>
       <c r="C228" s="28"/>
@@ -8126,10 +8126,10 @@
       <c r="E228" s="28"/>
       <c r="F228" s="28"/>
       <c r="G228" s="28" t="str">
-        <f>CONCATENATE("M 22 ",'Elimination Matches'!O87)</f>
+        <f>'data'!$B$76</f>
       </c>
       <c r="I228" s="28" t="str">
-        <f>'data'!$B$79</f>
+        <f>CONCATENATE("M 23 ",'Elimination Matches'!G95)</f>
       </c>
       <c r="J228" s="28"/>
       <c r="K228" s="28"/>
@@ -8137,7 +8137,7 @@
       <c r="M228" s="28"/>
       <c r="N228" s="28"/>
       <c r="O228" s="28" t="str">
-        <f>CONCATENATE("M 23 ",'Elimination Matches'!G95)</f>
+        <f>'data'!$B$79</f>
       </c>
     </row>
     <row r="230">
@@ -8181,28 +8181,28 @@
       <c r="O234" s="20"/>
     </row>
     <row r="235">
-      <c r="A235" s="29" t="s">
+      <c r="A235" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D235" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G235" s="30" t="s">
+      <c r="G235" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I235" s="29" t="s">
+      <c r="I235" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L235" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O235" s="30" t="s">
+      <c r="O235" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="28" t="str">
-        <f>'data'!$B$82</f>
+        <f>CONCATENATE("M 24 ",'Elimination Matches'!O95)</f>
       </c>
       <c r="B236" s="28"/>
       <c r="C236" s="28"/>
@@ -8210,10 +8210,10 @@
       <c r="E236" s="28"/>
       <c r="F236" s="28"/>
       <c r="G236" s="28" t="str">
-        <f>CONCATENATE("M 24 ",'Elimination Matches'!O95)</f>
+        <f>'data'!$B$82</f>
       </c>
       <c r="I236" s="28" t="str">
-        <f>'data'!$B$85</f>
+        <f>CONCATENATE("M 25 ",'Elimination Matches'!G103)</f>
       </c>
       <c r="J236" s="28"/>
       <c r="K236" s="28"/>
@@ -8221,7 +8221,7 @@
       <c r="M236" s="28"/>
       <c r="N236" s="28"/>
       <c r="O236" s="28" t="str">
-        <f>CONCATENATE("M 25 ",'Elimination Matches'!G103)</f>
+        <f>'data'!$B$85</f>
       </c>
     </row>
     <row r="238">
@@ -8265,28 +8265,28 @@
       <c r="O242" s="20"/>
     </row>
     <row r="243">
-      <c r="A243" s="29" t="s">
+      <c r="A243" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D243" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G243" s="30" t="s">
+      <c r="G243" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I243" s="29" t="s">
+      <c r="I243" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L243" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O243" s="30" t="s">
+      <c r="O243" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="28" t="str">
-        <f>'data'!$B$88</f>
+        <f>CONCATENATE("M 26 ",'Elimination Matches'!O103)</f>
       </c>
       <c r="B244" s="28"/>
       <c r="C244" s="28"/>
@@ -8294,10 +8294,10 @@
       <c r="E244" s="28"/>
       <c r="F244" s="28"/>
       <c r="G244" s="28" t="str">
-        <f>CONCATENATE("M 26 ",'Elimination Matches'!O103)</f>
+        <f>'data'!$B$88</f>
       </c>
       <c r="I244" s="28" t="str">
-        <f>'data'!$B$91</f>
+        <f>CONCATENATE("M 27 ",'Elimination Matches'!G111)</f>
       </c>
       <c r="J244" s="28"/>
       <c r="K244" s="28"/>
@@ -8305,7 +8305,7 @@
       <c r="M244" s="28"/>
       <c r="N244" s="28"/>
       <c r="O244" s="28" t="str">
-        <f>CONCATENATE("M 27 ",'Elimination Matches'!G111)</f>
+        <f>'data'!$B$91</f>
       </c>
     </row>
     <row r="246">
@@ -8368,28 +8368,28 @@
       <c r="O257" s="20"/>
     </row>
     <row r="258">
-      <c r="A258" s="29" t="s">
+      <c r="A258" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D258" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G258" s="30" t="s">
+      <c r="G258" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I258" s="29" t="s">
+      <c r="I258" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L258" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O258" s="30" t="s">
+      <c r="O258" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="28" t="str">
-        <f>CONCATENATE("M 28 ",'Elimination Matches'!G126)</f>
+        <f>CONCATENATE("M 29 ",'Elimination Matches'!O126)</f>
       </c>
       <c r="B259" s="28"/>
       <c r="C259" s="28"/>
@@ -8397,10 +8397,10 @@
       <c r="E259" s="28"/>
       <c r="F259" s="28"/>
       <c r="G259" s="28" t="str">
-        <f>CONCATENATE("M 29 ",'Elimination Matches'!O126)</f>
+        <f>CONCATENATE("M 28 ",'Elimination Matches'!G126)</f>
       </c>
       <c r="I259" s="28" t="str">
-        <f>CONCATENATE("M 30 ",'Elimination Matches'!G134)</f>
+        <f>CONCATENATE("M 31 ",'Elimination Matches'!O134)</f>
       </c>
       <c r="J259" s="28"/>
       <c r="K259" s="28"/>
@@ -8408,7 +8408,7 @@
       <c r="M259" s="28"/>
       <c r="N259" s="28"/>
       <c r="O259" s="28" t="str">
-        <f>CONCATENATE("M 31 ",'Elimination Matches'!O134)</f>
+        <f>CONCATENATE("M 30 ",'Elimination Matches'!G134)</f>
       </c>
     </row>
     <row r="261">
@@ -8452,28 +8452,28 @@
       <c r="O265" s="20"/>
     </row>
     <row r="266">
-      <c r="A266" s="29" t="s">
+      <c r="A266" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D266" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G266" s="30" t="s">
+      <c r="G266" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I266" s="29" t="s">
+      <c r="I266" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L266" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O266" s="30" t="s">
+      <c r="O266" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="28" t="str">
-        <f>CONCATENATE("M 32 ",'Elimination Matches'!G142)</f>
+        <f>CONCATENATE("M 33 ",'Elimination Matches'!O142)</f>
       </c>
       <c r="B267" s="28"/>
       <c r="C267" s="28"/>
@@ -8481,10 +8481,10 @@
       <c r="E267" s="28"/>
       <c r="F267" s="28"/>
       <c r="G267" s="28" t="str">
-        <f>CONCATENATE("M 33 ",'Elimination Matches'!O142)</f>
+        <f>CONCATENATE("M 32 ",'Elimination Matches'!G142)</f>
       </c>
       <c r="I267" s="28" t="str">
-        <f>CONCATENATE("M 34 ",'Elimination Matches'!G150)</f>
+        <f>CONCATENATE("M 35 ",'Elimination Matches'!O150)</f>
       </c>
       <c r="J267" s="28"/>
       <c r="K267" s="28"/>
@@ -8492,7 +8492,7 @@
       <c r="M267" s="28"/>
       <c r="N267" s="28"/>
       <c r="O267" s="28" t="str">
-        <f>CONCATENATE("M 35 ",'Elimination Matches'!O150)</f>
+        <f>CONCATENATE("M 34 ",'Elimination Matches'!G150)</f>
       </c>
     </row>
     <row r="269">
@@ -8536,28 +8536,28 @@
       <c r="O273" s="20"/>
     </row>
     <row r="274">
-      <c r="A274" s="29" t="s">
+      <c r="A274" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D274" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G274" s="30" t="s">
+      <c r="G274" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I274" s="29" t="s">
+      <c r="I274" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L274" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O274" s="30" t="s">
+      <c r="O274" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="28" t="str">
-        <f>CONCATENATE("M 36 ",'Elimination Matches'!G158)</f>
+        <f>CONCATENATE("M 37 ",'Elimination Matches'!O158)</f>
       </c>
       <c r="B275" s="28"/>
       <c r="C275" s="28"/>
@@ -8565,10 +8565,10 @@
       <c r="E275" s="28"/>
       <c r="F275" s="28"/>
       <c r="G275" s="28" t="str">
-        <f>CONCATENATE("M 37 ",'Elimination Matches'!O158)</f>
+        <f>CONCATENATE("M 36 ",'Elimination Matches'!G158)</f>
       </c>
       <c r="I275" s="28" t="str">
-        <f>CONCATENATE("M 38 ",'Elimination Matches'!G166)</f>
+        <f>CONCATENATE("M 39 ",'Elimination Matches'!O166)</f>
       </c>
       <c r="J275" s="28"/>
       <c r="K275" s="28"/>
@@ -8576,7 +8576,7 @@
       <c r="M275" s="28"/>
       <c r="N275" s="28"/>
       <c r="O275" s="28" t="str">
-        <f>CONCATENATE("M 39 ",'Elimination Matches'!O166)</f>
+        <f>CONCATENATE("M 38 ",'Elimination Matches'!G166)</f>
       </c>
     </row>
     <row r="277">
@@ -8620,28 +8620,28 @@
       <c r="O281" s="20"/>
     </row>
     <row r="282">
-      <c r="A282" s="29" t="s">
+      <c r="A282" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D282" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G282" s="30" t="s">
+      <c r="G282" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I282" s="29" t="s">
+      <c r="I282" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L282" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O282" s="30" t="s">
+      <c r="O282" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="28" t="str">
-        <f>CONCATENATE("M 40 ",'Elimination Matches'!G174)</f>
+        <f>CONCATENATE("M 41 ",'Elimination Matches'!O174)</f>
       </c>
       <c r="B283" s="28"/>
       <c r="C283" s="28"/>
@@ -8649,10 +8649,10 @@
       <c r="E283" s="28"/>
       <c r="F283" s="28"/>
       <c r="G283" s="28" t="str">
-        <f>CONCATENATE("M 41 ",'Elimination Matches'!O174)</f>
+        <f>CONCATENATE("M 40 ",'Elimination Matches'!G174)</f>
       </c>
       <c r="I283" s="28" t="str">
-        <f>CONCATENATE("M 42 ",'Elimination Matches'!G182)</f>
+        <f>CONCATENATE("M 43 ",'Elimination Matches'!O182)</f>
       </c>
       <c r="J283" s="28"/>
       <c r="K283" s="28"/>
@@ -8660,7 +8660,7 @@
       <c r="M283" s="28"/>
       <c r="N283" s="28"/>
       <c r="O283" s="28" t="str">
-        <f>CONCATENATE("M 43 ",'Elimination Matches'!O182)</f>
+        <f>CONCATENATE("M 42 ",'Elimination Matches'!G182)</f>
       </c>
     </row>
     <row r="285">
@@ -8704,28 +8704,28 @@
       <c r="O289" s="20"/>
     </row>
     <row r="290">
-      <c r="A290" s="29" t="s">
+      <c r="A290" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D290" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G290" s="30" t="s">
+      <c r="G290" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I290" s="29" t="s">
+      <c r="I290" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L290" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O290" s="30" t="s">
+      <c r="O290" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="28" t="str">
-        <f>CONCATENATE("M 44 ",'Elimination Matches'!G190)</f>
+        <f>CONCATENATE("M 45 ",'Elimination Matches'!O190)</f>
       </c>
       <c r="B291" s="28"/>
       <c r="C291" s="28"/>
@@ -8733,10 +8733,10 @@
       <c r="E291" s="28"/>
       <c r="F291" s="28"/>
       <c r="G291" s="28" t="str">
-        <f>CONCATENATE("M 45 ",'Elimination Matches'!O190)</f>
+        <f>CONCATENATE("M 44 ",'Elimination Matches'!G190)</f>
       </c>
       <c r="I291" s="28" t="str">
-        <f>CONCATENATE("M 46 ",'Elimination Matches'!G198)</f>
+        <f>CONCATENATE("M 47 ",'Elimination Matches'!O198)</f>
       </c>
       <c r="J291" s="28"/>
       <c r="K291" s="28"/>
@@ -8744,7 +8744,7 @@
       <c r="M291" s="28"/>
       <c r="N291" s="28"/>
       <c r="O291" s="28" t="str">
-        <f>CONCATENATE("M 47 ",'Elimination Matches'!O198)</f>
+        <f>CONCATENATE("M 46 ",'Elimination Matches'!G198)</f>
       </c>
     </row>
     <row r="293">
@@ -8788,28 +8788,28 @@
       <c r="O297" s="20"/>
     </row>
     <row r="298">
-      <c r="A298" s="29" t="s">
+      <c r="A298" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D298" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G298" s="30" t="s">
+      <c r="G298" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I298" s="29" t="s">
+      <c r="I298" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L298" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O298" s="30" t="s">
+      <c r="O298" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="28" t="str">
-        <f>CONCATENATE("M 48 ",'Elimination Matches'!G206)</f>
+        <f>CONCATENATE("M 49 ",'Elimination Matches'!O206)</f>
       </c>
       <c r="B299" s="28"/>
       <c r="C299" s="28"/>
@@ -8817,10 +8817,10 @@
       <c r="E299" s="28"/>
       <c r="F299" s="28"/>
       <c r="G299" s="28" t="str">
-        <f>CONCATENATE("M 49 ",'Elimination Matches'!O206)</f>
+        <f>CONCATENATE("M 48 ",'Elimination Matches'!G206)</f>
       </c>
       <c r="I299" s="28" t="str">
-        <f>CONCATENATE("M 50 ",'Elimination Matches'!G214)</f>
+        <f>CONCATENATE("M 51 ",'Elimination Matches'!O214)</f>
       </c>
       <c r="J299" s="28"/>
       <c r="K299" s="28"/>
@@ -8828,7 +8828,7 @@
       <c r="M299" s="28"/>
       <c r="N299" s="28"/>
       <c r="O299" s="28" t="str">
-        <f>CONCATENATE("M 51 ",'Elimination Matches'!O214)</f>
+        <f>CONCATENATE("M 50 ",'Elimination Matches'!G214)</f>
       </c>
     </row>
     <row r="301">
@@ -8872,28 +8872,28 @@
       <c r="O305" s="20"/>
     </row>
     <row r="306">
-      <c r="A306" s="29" t="s">
+      <c r="A306" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D306" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G306" s="30" t="s">
+      <c r="G306" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I306" s="29" t="s">
+      <c r="I306" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L306" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O306" s="30" t="s">
+      <c r="O306" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="28" t="str">
-        <f>CONCATENATE("M 52 ",'Elimination Matches'!G222)</f>
+        <f>CONCATENATE("M 53 ",'Elimination Matches'!O222)</f>
       </c>
       <c r="B307" s="28"/>
       <c r="C307" s="28"/>
@@ -8901,10 +8901,10 @@
       <c r="E307" s="28"/>
       <c r="F307" s="28"/>
       <c r="G307" s="28" t="str">
-        <f>CONCATENATE("M 53 ",'Elimination Matches'!O222)</f>
+        <f>CONCATENATE("M 52 ",'Elimination Matches'!G222)</f>
       </c>
       <c r="I307" s="28" t="str">
-        <f>CONCATENATE("M 54 ",'Elimination Matches'!G230)</f>
+        <f>CONCATENATE("M 55 ",'Elimination Matches'!O230)</f>
       </c>
       <c r="J307" s="28"/>
       <c r="K307" s="28"/>
@@ -8912,7 +8912,7 @@
       <c r="M307" s="28"/>
       <c r="N307" s="28"/>
       <c r="O307" s="28" t="str">
-        <f>CONCATENATE("M 55 ",'Elimination Matches'!O230)</f>
+        <f>CONCATENATE("M 54 ",'Elimination Matches'!G230)</f>
       </c>
     </row>
     <row r="309">
@@ -8956,28 +8956,28 @@
       <c r="O313" s="20"/>
     </row>
     <row r="314">
-      <c r="A314" s="29" t="s">
+      <c r="A314" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D314" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G314" s="30" t="s">
+      <c r="G314" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I314" s="29" t="s">
+      <c r="I314" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L314" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O314" s="30" t="s">
+      <c r="O314" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="28" t="str">
-        <f>CONCATENATE("M 56 ",'Elimination Matches'!G238)</f>
+        <f>CONCATENATE("M 57 ",'Elimination Matches'!O238)</f>
       </c>
       <c r="B315" s="28"/>
       <c r="C315" s="28"/>
@@ -8985,10 +8985,10 @@
       <c r="E315" s="28"/>
       <c r="F315" s="28"/>
       <c r="G315" s="28" t="str">
-        <f>CONCATENATE("M 57 ",'Elimination Matches'!O238)</f>
+        <f>CONCATENATE("M 56 ",'Elimination Matches'!G238)</f>
       </c>
       <c r="I315" s="28" t="str">
-        <f>CONCATENATE("M 58 ",'Elimination Matches'!G246)</f>
+        <f>CONCATENATE("M 59 ",'Elimination Matches'!O246)</f>
       </c>
       <c r="J315" s="28"/>
       <c r="K315" s="28"/>
@@ -8996,7 +8996,7 @@
       <c r="M315" s="28"/>
       <c r="N315" s="28"/>
       <c r="O315" s="28" t="str">
-        <f>CONCATENATE("M 59 ",'Elimination Matches'!O246)</f>
+        <f>CONCATENATE("M 58 ",'Elimination Matches'!G246)</f>
       </c>
     </row>
     <row r="317">
@@ -9059,28 +9059,28 @@
       <c r="O328" s="20"/>
     </row>
     <row r="329">
-      <c r="A329" s="29" t="s">
+      <c r="A329" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D329" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G329" s="30" t="s">
+      <c r="G329" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I329" s="29" t="s">
+      <c r="I329" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L329" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O329" s="30" t="s">
+      <c r="O329" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="28" t="str">
-        <f>CONCATENATE("M 60 ",'Elimination Matches'!G261)</f>
+        <f>CONCATENATE("M 61 ",'Elimination Matches'!O261)</f>
       </c>
       <c r="B330" s="28"/>
       <c r="C330" s="28"/>
@@ -9088,10 +9088,10 @@
       <c r="E330" s="28"/>
       <c r="F330" s="28"/>
       <c r="G330" s="28" t="str">
-        <f>CONCATENATE("M 61 ",'Elimination Matches'!O261)</f>
+        <f>CONCATENATE("M 60 ",'Elimination Matches'!G261)</f>
       </c>
       <c r="I330" s="28" t="str">
-        <f>CONCATENATE("M 62 ",'Elimination Matches'!G269)</f>
+        <f>CONCATENATE("M 63 ",'Elimination Matches'!O269)</f>
       </c>
       <c r="J330" s="28"/>
       <c r="K330" s="28"/>
@@ -9099,7 +9099,7 @@
       <c r="M330" s="28"/>
       <c r="N330" s="28"/>
       <c r="O330" s="28" t="str">
-        <f>CONCATENATE("M 63 ",'Elimination Matches'!O269)</f>
+        <f>CONCATENATE("M 62 ",'Elimination Matches'!G269)</f>
       </c>
     </row>
     <row r="332">
@@ -9143,28 +9143,28 @@
       <c r="O336" s="20"/>
     </row>
     <row r="337">
-      <c r="A337" s="29" t="s">
+      <c r="A337" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D337" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G337" s="30" t="s">
+      <c r="G337" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I337" s="29" t="s">
+      <c r="I337" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L337" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O337" s="30" t="s">
+      <c r="O337" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="28" t="str">
-        <f>CONCATENATE("M 64 ",'Elimination Matches'!G277)</f>
+        <f>CONCATENATE("M 65 ",'Elimination Matches'!O277)</f>
       </c>
       <c r="B338" s="28"/>
       <c r="C338" s="28"/>
@@ -9172,10 +9172,10 @@
       <c r="E338" s="28"/>
       <c r="F338" s="28"/>
       <c r="G338" s="28" t="str">
-        <f>CONCATENATE("M 65 ",'Elimination Matches'!O277)</f>
+        <f>CONCATENATE("M 64 ",'Elimination Matches'!G277)</f>
       </c>
       <c r="I338" s="28" t="str">
-        <f>CONCATENATE("M 66 ",'Elimination Matches'!G285)</f>
+        <f>CONCATENATE("M 67 ",'Elimination Matches'!O285)</f>
       </c>
       <c r="J338" s="28"/>
       <c r="K338" s="28"/>
@@ -9183,7 +9183,7 @@
       <c r="M338" s="28"/>
       <c r="N338" s="28"/>
       <c r="O338" s="28" t="str">
-        <f>CONCATENATE("M 67 ",'Elimination Matches'!O285)</f>
+        <f>CONCATENATE("M 66 ",'Elimination Matches'!G285)</f>
       </c>
     </row>
     <row r="340">
@@ -9227,28 +9227,28 @@
       <c r="O344" s="20"/>
     </row>
     <row r="345">
-      <c r="A345" s="29" t="s">
+      <c r="A345" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D345" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G345" s="30" t="s">
+      <c r="G345" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I345" s="29" t="s">
+      <c r="I345" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L345" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O345" s="30" t="s">
+      <c r="O345" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="28" t="str">
-        <f>CONCATENATE("M 68 ",'Elimination Matches'!G293)</f>
+        <f>CONCATENATE("M 69 ",'Elimination Matches'!O293)</f>
       </c>
       <c r="B346" s="28"/>
       <c r="C346" s="28"/>
@@ -9256,10 +9256,10 @@
       <c r="E346" s="28"/>
       <c r="F346" s="28"/>
       <c r="G346" s="28" t="str">
-        <f>CONCATENATE("M 69 ",'Elimination Matches'!O293)</f>
+        <f>CONCATENATE("M 68 ",'Elimination Matches'!G293)</f>
       </c>
       <c r="I346" s="28" t="str">
-        <f>CONCATENATE("M 70 ",'Elimination Matches'!G301)</f>
+        <f>CONCATENATE("M 71 ",'Elimination Matches'!O301)</f>
       </c>
       <c r="J346" s="28"/>
       <c r="K346" s="28"/>
@@ -9267,7 +9267,7 @@
       <c r="M346" s="28"/>
       <c r="N346" s="28"/>
       <c r="O346" s="28" t="str">
-        <f>CONCATENATE("M 71 ",'Elimination Matches'!O301)</f>
+        <f>CONCATENATE("M 70 ",'Elimination Matches'!G301)</f>
       </c>
     </row>
     <row r="348">
@@ -9311,28 +9311,28 @@
       <c r="O352" s="20"/>
     </row>
     <row r="353">
-      <c r="A353" s="29" t="s">
+      <c r="A353" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D353" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G353" s="30" t="s">
+      <c r="G353" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I353" s="29" t="s">
+      <c r="I353" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L353" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O353" s="30" t="s">
+      <c r="O353" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="28" t="str">
-        <f>CONCATENATE("M 72 ",'Elimination Matches'!G309)</f>
+        <f>CONCATENATE("M 73 ",'Elimination Matches'!O309)</f>
       </c>
       <c r="B354" s="28"/>
       <c r="C354" s="28"/>
@@ -9340,10 +9340,10 @@
       <c r="E354" s="28"/>
       <c r="F354" s="28"/>
       <c r="G354" s="28" t="str">
-        <f>CONCATENATE("M 73 ",'Elimination Matches'!O309)</f>
+        <f>CONCATENATE("M 72 ",'Elimination Matches'!G309)</f>
       </c>
       <c r="I354" s="28" t="str">
-        <f>CONCATENATE("M 74 ",'Elimination Matches'!G317)</f>
+        <f>CONCATENATE("M 75 ",'Elimination Matches'!O317)</f>
       </c>
       <c r="J354" s="28"/>
       <c r="K354" s="28"/>
@@ -9351,7 +9351,7 @@
       <c r="M354" s="28"/>
       <c r="N354" s="28"/>
       <c r="O354" s="28" t="str">
-        <f>CONCATENATE("M 75 ",'Elimination Matches'!O317)</f>
+        <f>CONCATENATE("M 74 ",'Elimination Matches'!G317)</f>
       </c>
     </row>
     <row r="356">
@@ -9414,28 +9414,28 @@
       <c r="O367" s="20"/>
     </row>
     <row r="368">
-      <c r="A368" s="29" t="s">
+      <c r="A368" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D368" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G368" s="30" t="s">
+      <c r="G368" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I368" s="29" t="s">
+      <c r="I368" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L368" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O368" s="30" t="s">
+      <c r="O368" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="28" t="str">
-        <f>CONCATENATE("M 76 ",'Elimination Matches'!G332)</f>
+        <f>CONCATENATE("M 77 ",'Elimination Matches'!O332)</f>
       </c>
       <c r="B369" s="28"/>
       <c r="C369" s="28"/>
@@ -9443,10 +9443,10 @@
       <c r="E369" s="28"/>
       <c r="F369" s="28"/>
       <c r="G369" s="28" t="str">
-        <f>CONCATENATE("M 77 ",'Elimination Matches'!O332)</f>
+        <f>CONCATENATE("M 76 ",'Elimination Matches'!G332)</f>
       </c>
       <c r="I369" s="28" t="str">
-        <f>CONCATENATE("M 78 ",'Elimination Matches'!G340)</f>
+        <f>CONCATENATE("M 79 ",'Elimination Matches'!O340)</f>
       </c>
       <c r="J369" s="28"/>
       <c r="K369" s="28"/>
@@ -9454,7 +9454,7 @@
       <c r="M369" s="28"/>
       <c r="N369" s="28"/>
       <c r="O369" s="28" t="str">
-        <f>CONCATENATE("M 79 ",'Elimination Matches'!O340)</f>
+        <f>CONCATENATE("M 78 ",'Elimination Matches'!G340)</f>
       </c>
     </row>
     <row r="371">
@@ -9498,28 +9498,28 @@
       <c r="O375" s="20"/>
     </row>
     <row r="376">
-      <c r="A376" s="29" t="s">
+      <c r="A376" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D376" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G376" s="30" t="s">
+      <c r="G376" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I376" s="29" t="s">
+      <c r="I376" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L376" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O376" s="30" t="s">
+      <c r="O376" s="29" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="28" t="str">
-        <f>CONCATENATE("M 80 ",'Elimination Matches'!G348)</f>
+        <f>CONCATENATE("M 81 ",'Elimination Matches'!O348)</f>
       </c>
       <c r="B377" s="28"/>
       <c r="C377" s="28"/>
@@ -9527,10 +9527,10 @@
       <c r="E377" s="28"/>
       <c r="F377" s="28"/>
       <c r="G377" s="28" t="str">
-        <f>CONCATENATE("M 81 ",'Elimination Matches'!O348)</f>
+        <f>CONCATENATE("M 80 ",'Elimination Matches'!G348)</f>
       </c>
       <c r="I377" s="28" t="str">
-        <f>CONCATENATE("M 82 ",'Elimination Matches'!G356)</f>
+        <f>CONCATENATE("M 83 ",'Elimination Matches'!O356)</f>
       </c>
       <c r="J377" s="28"/>
       <c r="K377" s="28"/>
@@ -9538,7 +9538,7 @@
       <c r="M377" s="28"/>
       <c r="N377" s="28"/>
       <c r="O377" s="28" t="str">
-        <f>CONCATENATE("M 83 ",'Elimination Matches'!O356)</f>
+        <f>CONCATENATE("M 82 ",'Elimination Matches'!G356)</f>
       </c>
     </row>
     <row r="379">
@@ -9601,22 +9601,22 @@
       <c r="O390" s="20"/>
     </row>
     <row r="391">
-      <c r="A391" s="29" t="s">
+      <c r="A391" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D391" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G391" s="30" t="s">
+      <c r="G391" s="29" t="s">
         <v>211</v>
       </c>
-      <c r="I391" s="29" t="s">
+      <c r="I391" s="30" t="s">
         <v>209</v>
       </c>
       <c r="L391" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="O391" s="30" t="s">
+      <c r="O391" s="29" t="s">
         <v>211</v>
       </c>
     </row>
@@ -9695,13 +9695,13 @@
       <c r="G405" s="20"/>
     </row>
     <row r="406">
-      <c r="A406" s="29" t="s">
+      <c r="A406" s="30" t="s">
         <v>209</v>
       </c>
       <c r="D406" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G406" s="30" t="s">
+      <c r="G406" s="29" t="s">
         <v>211</v>
       </c>
     </row>

</xml_diff>